<commit_message>
feat(poa-rendicion): aprobar POA Presupuestal aprueba rendiciones y descuenta saldo (item 6)
- PoaController::aprobar -> Rendicion::aprobarPorPrograma(): al aprobar el POA Presupuestal, las rendiciones del programa pasan a Aprobada (estado=1) y se congelan.
- RendicionController::crear: adenda del Contador sobre POA ya Aprobado nace Aprobada.
- Rendicion: constantes PENDIENTE/APROBADA + aprobarPorPrograma() (UPDATE directo, estado fuera de columnasDB para que el CRUD no lo toque).
- migr. 018: vistas de saldo contable restan solo rendiciones estado=1.
- migr. 019: backfill de rendiciones de programas con POA ya Aprobado (idempotente).
- UI: banner en poa/admin + confirmacion en poa/revisar avisan del descuento.
- QA: qa_poa_presupuestal.ps1 ahora 21/21 (rendicion no mueve saldo hasta aprobar).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/views/reporte/storage/reports/reporte_poa_ADMN.xlsx
+++ b/views/reporte/storage/reports/reporte_poa_ADMN.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
   <si>
     <t>PROCESO DE PROYECTOS</t>
   </si>
@@ -63,6 +63,18 @@
   </si>
   <si>
     <t>MOBILIARIO</t>
+  </si>
+  <si>
+    <t>PRESUPUESTO - 2026 - PROGRAMA PROGRAMA DEMO 2</t>
+  </si>
+  <si>
+    <t>PRO01 PRODUCTO 1</t>
+  </si>
+  <si>
+    <t>ACT01 ACTIVIDAD 01</t>
+  </si>
+  <si>
+    <t>RUBRO 01</t>
   </si>
 </sst>
 </file>
@@ -112,7 +124,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -122,6 +134,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF5733"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -138,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
@@ -152,8 +170,14 @@
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
@@ -198,6 +222,36 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="0"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="476250" cy="381000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -504,7 +558,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="true" style="0"/>
@@ -535,14 +589,14 @@
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
     </row>
     <row r="3" spans="1:9" customHeight="1" ht="15">
       <c r="A3" s="4"/>
@@ -562,16 +616,16 @@
     <row r="4" spans="1:9" customHeight="1" ht="52">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -592,16 +646,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="7"/>
+      <c r="D5" s="9"/>
       <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>3500.0</v>
       </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" spans="1:9" customHeight="1" ht="53">
       <c r="A6" s="2"/>
@@ -609,18 +663,18 @@
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="9">
         <v>12000.0</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7">
+      <c r="F6" s="9"/>
+      <c r="G6" s="9">
         <v>15500.0</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="9">
         <v>4133.33</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="9">
         <v>3827.16</v>
       </c>
     </row>
@@ -630,16 +684,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="7"/>
+      <c r="D7" s="9"/>
       <c r="E7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="9">
         <v>4500.0</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
     </row>
     <row r="8" spans="1:9" customHeight="1" ht="53">
       <c r="A8" s="2"/>
@@ -647,18 +701,18 @@
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="9">
         <v>8000.0</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7">
+      <c r="F8" s="9"/>
+      <c r="G8" s="9">
         <v>12500.0</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="9">
         <v>3333.33</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="9">
         <v>3086.42</v>
       </c>
     </row>
@@ -666,26 +720,165 @@
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="8">
+      <c r="D9" s="10">
         <f>SUM(D5:D8)</f>
         <v>20000</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="8">
+      <c r="F9" s="10">
         <f>SUM(F5:F8)</f>
         <v>8000</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="10">
         <f>SUM(G5:G8)</f>
         <v>28000</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="11">
         <f>SUM(H5:H8)</f>
         <v>7466.66</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="12">
         <f>SUM(I5:I8)</f>
         <v>6913.58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" customHeight="1" ht="35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" customHeight="1" ht="53">
+      <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="9">
+        <v>4500.0</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9">
+        <v>4500.0</v>
+      </c>
+      <c r="H16" s="9">
+        <v>1200.0</v>
+      </c>
+      <c r="I16" s="9">
+        <v>1111.11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="10">
+        <f>SUM(D16:D16)</f>
+        <v>4500</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="10">
+        <f>SUM(F16:F16)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="10">
+        <f>SUM(G16:G16)</f>
+        <v>4500</v>
+      </c>
+      <c r="H17" s="11">
+        <f>SUM(H16:H16)</f>
+        <v>1200</v>
+      </c>
+      <c r="I17" s="12">
+        <f>SUM(I16:I16)</f>
+        <v>1111.11</v>
       </c>
     </row>
   </sheetData>
@@ -694,6 +887,10 @@
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="E3:F3"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B7:B8"/>

</xml_diff>